<commit_message>
Works for Vorm 1 & 2 Cp
</commit_message>
<xml_diff>
--- a/data/IPT_Tabel_B2.xlsx
+++ b/data/IPT_Tabel_B2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elise\Documents\Code_Projects\IPT_Work\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elise\Documents\Code_Projects\IPT_Work\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BD32213-1F74-4EBE-88B5-ACF16100B6BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7341B35-7C71-4113-BED2-403468F8AA04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="852" yWindow="936" windowWidth="18984" windowHeight="11304" xr2:uid="{336C27D0-6682-4DCC-A3BE-8962172894D3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{336C27D0-6682-4DCC-A3BE-8962172894D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="686" uniqueCount="457">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="452">
   <si>
     <t>Stofnaam (NL)</t>
   </si>
@@ -644,30 +644,6 @@
   </si>
   <si>
     <r>
-      <t>-8.66 • 10</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="7"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t> </t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>Calciumcarbonaat</t>
     </r>
     <r>
@@ -727,30 +703,6 @@
   </si>
   <si>
     <t>4.975 </t>
-  </si>
-  <si>
-    <r>
-      <t>-12.87 • 10</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="7"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t> </t>
-    </r>
   </si>
   <si>
     <r>
@@ -1970,30 +1922,6 @@
   </si>
   <si>
     <r>
-      <t>-17.72 • 10</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="7"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t> </t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>Koolstof</t>
     </r>
     <r>
@@ -2045,30 +1973,6 @@
   </si>
   <si>
     <r>
-      <t>-4.891 • 10</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="7"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t> </t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>Koolstofdioxide</t>
     </r>
     <r>
@@ -2398,30 +2302,6 @@
   </si>
   <si>
     <t>0.5008 </t>
-  </si>
-  <si>
-    <r>
-      <t>-8.732 • 10</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="7"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t> </t>
-    </r>
   </si>
   <si>
     <r>
@@ -4478,7 +4358,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4515,13 +4395,6 @@
     </font>
     <font>
       <sz val="9"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <vertAlign val="superscript"/>
-      <sz val="7"/>
-      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -4718,7 +4591,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="11" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5053,7 +4928,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89D9F275-69BE-481B-B5DA-385923738F5A}">
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:K68"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -5099,7 +4974,7 @@
         <v>15</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>454</v>
+        <v>449</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>16</v>
@@ -5130,7 +5005,7 @@
         <v>15</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>454</v>
+        <v>449</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>16</v>
@@ -5159,7 +5034,7 @@
     </row>
     <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
-        <v>456</v>
+        <v>451</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>27</v>
@@ -5385,23 +5260,23 @@
       <c r="I10" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="J10" s="1" t="s">
-        <v>75</v>
+      <c r="J10" s="15">
+        <v>-86600000000</v>
       </c>
       <c r="K10" s="5"/>
     </row>
     <row r="11" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>79</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>47</v>
@@ -5413,28 +5288,28 @@
         <v>48</v>
       </c>
       <c r="H11" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="I11" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="I11" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>82</v>
+      <c r="J11" s="15">
+        <v>-128700000000</v>
       </c>
       <c r="K11" s="5"/>
     </row>
     <row r="12" spans="1:11" ht="36" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="D12" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>86</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>47</v>
@@ -5446,7 +5321,7 @@
         <v>48</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
@@ -5454,16 +5329,16 @@
     </row>
     <row r="13" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="D13" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>22</v>
@@ -5475,30 +5350,30 @@
         <v>19</v>
       </c>
       <c r="H13" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="J13" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="K13" s="6" t="s">
         <v>93</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="K13" s="6" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="D14" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>22</v>
@@ -5510,30 +5385,30 @@
         <v>19</v>
       </c>
       <c r="H14" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="J14" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="K14" s="6" t="s">
         <v>101</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="K14" s="6" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C15" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="D15" s="14" t="s">
         <v>105</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="D15" s="14" t="s">
-        <v>107</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>17</v>
@@ -5545,30 +5420,30 @@
         <v>48</v>
       </c>
       <c r="H15" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="J15" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="I15" s="1" t="s">
+      <c r="K15" s="6" t="s">
         <v>109</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="K15" s="6" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C16" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="D16" s="14" t="s">
         <v>105</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>107</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>22</v>
@@ -5580,30 +5455,30 @@
         <v>19</v>
       </c>
       <c r="H16" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="J16" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="I16" s="1" t="s">
+      <c r="K16" s="6" t="s">
         <v>113</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="K16" s="6" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="D17" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>119</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>17</v>
@@ -5615,26 +5490,26 @@
         <v>30</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J17" s="1"/>
       <c r="K17" s="6"/>
     </row>
     <row r="18" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="D18" s="1" t="s">
         <v>123</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>125</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>22</v>
@@ -5646,30 +5521,30 @@
         <v>19</v>
       </c>
       <c r="H18" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="J18" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="K18" s="6" t="s">
         <v>127</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="K18" s="6" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C19" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="D19" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>133</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>22</v>
@@ -5681,30 +5556,30 @@
         <v>30</v>
       </c>
       <c r="H19" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="J19" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="I19" s="1" t="s">
+      <c r="K19" s="6" t="s">
         <v>135</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="K19" s="6" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="D20" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>141</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>22</v>
@@ -5716,28 +5591,28 @@
         <v>30</v>
       </c>
       <c r="H20" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="J20" s="1" t="s">
         <v>142</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>144</v>
       </c>
       <c r="K20" s="5"/>
     </row>
     <row r="21" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="C21" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="D21" s="1" t="s">
         <v>146</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>148</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>22</v>
@@ -5749,30 +5624,30 @@
         <v>30</v>
       </c>
       <c r="H21" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="J21" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="K21" s="6" t="s">
         <v>150</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="K21" s="6" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="C22" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="D22" s="14" t="s">
         <v>154</v>
-      </c>
-      <c r="C22" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="D22" s="14" t="s">
-        <v>156</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>17</v>
@@ -5784,7 +5659,7 @@
         <v>19</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
@@ -5792,16 +5667,16 @@
     </row>
     <row r="23" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="C23" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="D23" s="14" t="s">
         <v>154</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="D23" s="14" t="s">
-        <v>156</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>22</v>
@@ -5813,30 +5688,30 @@
         <v>19</v>
       </c>
       <c r="H23" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="J23" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="I23" s="1" t="s">
+      <c r="K23" s="6" t="s">
         <v>159</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="K23" s="6" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="D24" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>165</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>22</v>
@@ -5848,30 +5723,30 @@
         <v>19</v>
       </c>
       <c r="H24" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="J24" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="I24" s="1" t="s">
+      <c r="K24" s="6" t="s">
         <v>167</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="K24" s="6" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
-        <v>455</v>
+        <v>450</v>
       </c>
       <c r="B25" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>170</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>172</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>22</v>
@@ -5883,30 +5758,30 @@
         <v>19</v>
       </c>
       <c r="H25" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="J25" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="I25" s="1" t="s">
+      <c r="K25" s="6" t="s">
         <v>174</v>
-      </c>
-      <c r="J25" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="K25" s="6" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>179</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>22</v>
@@ -5918,7 +5793,7 @@
         <v>19</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
@@ -5926,16 +5801,16 @@
     </row>
     <row r="27" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="C27" s="13" t="s">
         <v>181</v>
       </c>
-      <c r="B27" s="13" t="s">
+      <c r="D27" s="14" t="s">
         <v>182</v>
-      </c>
-      <c r="C27" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="D27" s="14" t="s">
-        <v>184</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>17</v>
@@ -5947,7 +5822,7 @@
         <v>30</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
@@ -5955,16 +5830,16 @@
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="C28" s="13" t="s">
         <v>181</v>
       </c>
-      <c r="B28" s="13" t="s">
+      <c r="D28" s="14" t="s">
         <v>182</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="D28" s="14" t="s">
-        <v>184</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>22</v>
@@ -5976,30 +5851,30 @@
         <v>30</v>
       </c>
       <c r="H28" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="J28" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="I28" s="1" t="s">
+      <c r="K28" s="6" t="s">
         <v>187</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="K28" s="6" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="C29" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="D29" s="1" t="s">
         <v>191</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>193</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>47</v>
@@ -6011,28 +5886,28 @@
         <v>48</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>196</v>
+        <v>193</v>
+      </c>
+      <c r="J29" s="15">
+        <v>-177200000000</v>
       </c>
       <c r="K29" s="5"/>
     </row>
-    <row r="30" spans="1:11" ht="23.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>197</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>200</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>47</v>
@@ -6044,28 +5919,28 @@
         <v>48</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="J30" s="1" t="s">
-        <v>203</v>
+        <v>199</v>
+      </c>
+      <c r="J30" s="15">
+        <v>-48910000000</v>
       </c>
       <c r="K30" s="5"/>
     </row>
     <row r="31" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="7" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>22</v>
@@ -6077,30 +5952,30 @@
         <v>30</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="K31" s="6" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="7" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>22</v>
@@ -6112,30 +5987,30 @@
         <v>30</v>
       </c>
       <c r="H32" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="7" t="s">
         <v>216</v>
       </c>
-      <c r="I32" s="1" t="s">
+      <c r="B33" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="J32" s="1" t="s">
+      <c r="C33" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="K32" s="6" t="s">
+      <c r="D33" s="1" t="s">
         <v>219</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>223</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>47</v>
@@ -6147,24 +6022,24 @@
         <v>48</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="J33" s="2"/>
       <c r="K33" s="5"/>
     </row>
-    <row r="34" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="7" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="C34" s="4"/>
       <c r="D34" s="1" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>22</v>
@@ -6176,30 +6051,30 @@
         <v>30</v>
       </c>
       <c r="H34" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="J34" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="I34" s="1" t="s">
+      <c r="B35" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="J34" s="1" t="s">
+      <c r="C35" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="K34" s="6" t="s">
+      <c r="D35" s="1" t="s">
         <v>232</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>236</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>47</v>
@@ -6211,26 +6086,26 @@
         <v>48</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="J35" s="2"/>
       <c r="K35" s="5"/>
     </row>
-    <row r="36" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="7" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>47</v>
@@ -6242,28 +6117,28 @@
         <v>48</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="J36" s="1" t="s">
-        <v>245</v>
+        <v>240</v>
+      </c>
+      <c r="J36" s="15">
+        <v>-87320000000</v>
       </c>
       <c r="K36" s="5"/>
     </row>
-    <row r="37" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="7" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>22</v>
@@ -6275,31 +6150,30 @@
         <v>19</v>
       </c>
       <c r="H37" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="B38" s="13" t="s">
         <v>250</v>
       </c>
-      <c r="I37" s="1" t="s">
+      <c r="C38" s="13" t="s">
         <v>251</v>
       </c>
-      <c r="J37" s="1" t="s">
+      <c r="D38" s="14" t="s">
         <v>252</v>
-      </c>
-      <c r="K37" s="6" t="s">
-        <v>253</v>
-      </c>
-      <c r="L37" s="15"/>
-    </row>
-    <row r="38" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="12" t="s">
-        <v>254</v>
-      </c>
-      <c r="B38" s="13" t="s">
-        <v>255</v>
-      </c>
-      <c r="C38" s="13" t="s">
-        <v>256</v>
-      </c>
-      <c r="D38" s="14" t="s">
-        <v>257</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>17</v>
@@ -6311,26 +6185,26 @@
         <v>19</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J38" s="2"/>
       <c r="K38" s="5"/>
     </row>
-    <row r="39" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="12" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>22</v>
@@ -6342,30 +6216,30 @@
         <v>30</v>
       </c>
       <c r="H39" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="I39" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="J39" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="K39" s="6" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="36" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="B40" s="3" t="s">
         <v>260</v>
       </c>
-      <c r="I39" s="1" t="s">
+      <c r="C40" s="3" t="s">
         <v>261</v>
       </c>
-      <c r="J39" s="1" t="s">
+      <c r="D40" s="1" t="s">
         <v>262</v>
-      </c>
-      <c r="K39" s="6" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" ht="36" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="7" t="s">
-        <v>264</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>265</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>266</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>267</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>22</v>
@@ -6377,30 +6251,30 @@
         <v>19</v>
       </c>
       <c r="H40" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="I40" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="K40" s="6" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="B41" s="3" t="s">
         <v>268</v>
       </c>
-      <c r="I40" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="K40" s="6" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>273</v>
-      </c>
       <c r="C41" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>22</v>
@@ -6412,24 +6286,24 @@
         <v>19</v>
       </c>
       <c r="H41" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="J41" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="K41" s="6" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="B42" s="3" t="s">
         <v>274</v>
-      </c>
-      <c r="I41" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="J41" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="K41" s="6" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="7" t="s">
-        <v>278</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>279</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>62</v>
@@ -6447,30 +6321,30 @@
         <v>30</v>
       </c>
       <c r="H42" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="J42" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="K42" s="6" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="B43" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="I42" s="1" t="s">
+      <c r="C43" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="J42" s="1" t="s">
+      <c r="D43" s="1" t="s">
         <v>282</v>
-      </c>
-      <c r="K42" s="6" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="7" t="s">
-        <v>284</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>287</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>22</v>
@@ -6482,30 +6356,30 @@
         <v>30</v>
       </c>
       <c r="H43" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="J43" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="K43" s="6" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="B44" s="13" t="s">
         <v>288</v>
       </c>
-      <c r="I43" s="1" t="s">
+      <c r="C44" s="13" t="s">
         <v>289</v>
       </c>
-      <c r="J43" s="1" t="s">
+      <c r="D44" s="14" t="s">
         <v>290</v>
-      </c>
-      <c r="K43" s="6" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="12" t="s">
-        <v>292</v>
-      </c>
-      <c r="B44" s="13" t="s">
-        <v>293</v>
-      </c>
-      <c r="C44" s="13" t="s">
-        <v>294</v>
-      </c>
-      <c r="D44" s="14" t="s">
-        <v>295</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>17</v>
@@ -6517,26 +6391,26 @@
         <v>30</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="J44" s="2"/>
       <c r="K44" s="5"/>
     </row>
-    <row r="45" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A45" s="12" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>22</v>
@@ -6548,30 +6422,30 @@
         <v>30</v>
       </c>
       <c r="H45" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="J45" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="K45" s="6" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="B46" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="I45" s="1" t="s">
+      <c r="C46" s="3" t="s">
         <v>299</v>
       </c>
-      <c r="J45" s="1" t="s">
+      <c r="D46" s="1" t="s">
         <v>300</v>
-      </c>
-      <c r="K45" s="6" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>303</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>304</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>305</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>22</v>
@@ -6583,30 +6457,30 @@
         <v>30</v>
       </c>
       <c r="H46" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="K46" s="6" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="24" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="B47" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="I46" s="1" t="s">
+      <c r="C47" s="3" t="s">
         <v>307</v>
       </c>
-      <c r="J46" s="1" t="s">
+      <c r="D47" s="1" t="s">
         <v>308</v>
-      </c>
-      <c r="K46" s="6" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="7" t="s">
-        <v>310</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>311</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>312</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>313</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>22</v>
@@ -6618,30 +6492,30 @@
         <v>19</v>
       </c>
       <c r="H47" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="J47" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="K47" s="6" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="B48" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="I47" s="1" t="s">
+      <c r="C48" s="3" t="s">
         <v>315</v>
       </c>
-      <c r="J47" s="1" t="s">
+      <c r="D48" s="1" t="s">
         <v>316</v>
-      </c>
-      <c r="K47" s="6" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="7" t="s">
-        <v>318</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>320</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>321</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>17</v>
@@ -6653,7 +6527,7 @@
         <v>30</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
@@ -6661,16 +6535,16 @@
     </row>
     <row r="49" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A49" s="7" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>22</v>
@@ -6682,30 +6556,30 @@
         <v>30</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="I49" s="1" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="J49" s="1" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A50" s="7" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>22</v>
@@ -6717,30 +6591,30 @@
         <v>30</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="K50" s="6" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="7" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>22</v>
@@ -6752,30 +6626,30 @@
         <v>19</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="K51" s="6" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A52" s="7" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>17</v>
@@ -6787,26 +6661,26 @@
         <v>48</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="J52" s="2"/>
       <c r="K52" s="5"/>
     </row>
     <row r="53" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A53" s="7" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>47</v>
@@ -6818,7 +6692,7 @@
         <v>48</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
@@ -6826,22 +6700,22 @@
     </row>
     <row r="54" spans="1:11" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A54" s="7" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F54" s="1">
-        <v>1</v>
+      <c r="F54" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="G54" s="1" t="s">
         <v>12</v>
@@ -6855,13 +6729,13 @@
     </row>
     <row r="55" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="12" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="B55" s="13" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="C55" s="13" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="D55" s="14">
         <v>92.13</v>
@@ -6876,73 +6750,73 @@
         <v>19</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="J55" s="2"/>
       <c r="K55" s="5"/>
     </row>
     <row r="56" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A56" s="12" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="B56" s="13" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="D56" s="14" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F56" s="1">
-        <v>1</v>
+      <c r="F56" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="G56" s="1" t="s">
         <v>30</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="K56" s="6" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
     </row>
     <row r="57" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="12" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="B57" s="13" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="D57" s="14" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F57" s="1">
-        <v>1</v>
+      <c r="F57" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="G57" s="1" t="s">
         <v>30</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
@@ -6956,10 +6830,10 @@
         <v>13</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="D58" s="14" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>11</v>
@@ -6971,30 +6845,30 @@
         <v>30</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="K58" s="6" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
     </row>
     <row r="59" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A59" s="7" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>22</v>
@@ -7006,30 +6880,30 @@
         <v>19</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="K59" s="6" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
     </row>
     <row r="60" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A60" s="7" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>22</v>
@@ -7041,30 +6915,30 @@
         <v>19</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="K60" s="6" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
     </row>
     <row r="61" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A61" s="7" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>22</v>
@@ -7076,30 +6950,30 @@
         <v>19</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="K61" s="6" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A62" s="7" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>22</v>
@@ -7111,28 +6985,28 @@
         <v>19</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="K62" s="5"/>
     </row>
     <row r="63" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A63" s="7" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>22</v>
@@ -7144,30 +7018,30 @@
         <v>19</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>417</v>
+        <v>412</v>
       </c>
       <c r="K63" s="6" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
     </row>
     <row r="64" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A64" s="7" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>22</v>
@@ -7179,30 +7053,30 @@
         <v>30</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="I64" s="1" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="K64" s="6" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
     </row>
     <row r="65" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="7" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>47</v>
@@ -7214,26 +7088,26 @@
         <v>48</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="I65" s="1" t="s">
-        <v>431</v>
+        <v>426</v>
       </c>
       <c r="J65" s="2"/>
       <c r="K65" s="5"/>
     </row>
     <row r="66" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A66" s="7" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>17</v>
@@ -7245,26 +7119,26 @@
         <v>30</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>436</v>
+        <v>431</v>
       </c>
       <c r="I66" s="1" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="J66" s="2"/>
       <c r="K66" s="5"/>
     </row>
     <row r="67" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A67" s="7" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>439</v>
+        <v>434</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>441</v>
+        <v>436</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>22</v>
@@ -7276,51 +7150,51 @@
         <v>30</v>
       </c>
       <c r="H67" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="K67" s="6" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A68" s="8" t="s">
+        <v>441</v>
+      </c>
+      <c r="B68" s="9" t="s">
         <v>442</v>
       </c>
-      <c r="I67" s="1" t="s">
+      <c r="C68" s="9" t="s">
         <v>443</v>
       </c>
-      <c r="J67" s="1" t="s">
+      <c r="D68" s="10" t="s">
         <v>444</v>
-      </c>
-      <c r="K67" s="6" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" ht="24" x14ac:dyDescent="0.3">
-      <c r="A68" s="8" t="s">
-        <v>446</v>
-      </c>
-      <c r="B68" s="9" t="s">
-        <v>447</v>
-      </c>
-      <c r="C68" s="9" t="s">
-        <v>448</v>
-      </c>
-      <c r="D68" s="10" t="s">
-        <v>449</v>
       </c>
       <c r="E68" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="F68" s="10" t="s">
+      <c r="F68" s="1" t="s">
         <v>18</v>
       </c>
       <c r="G68" s="10" t="s">
         <v>30</v>
       </c>
       <c r="H68" s="10" t="s">
-        <v>450</v>
+        <v>445</v>
       </c>
       <c r="I68" s="10" t="s">
-        <v>451</v>
+        <v>446</v>
       </c>
       <c r="J68" s="10" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
       <c r="K68" s="11" t="s">
-        <v>453</v>
+        <v>448</v>
       </c>
     </row>
   </sheetData>

</xml_diff>